<commit_message>
Deploying to gh-pages from @ jariasca9/iuaf-pro-frontend@14ab8bd1db8c13dcb9d188dbee781fd5eac9d3b0 🚀
</commit_message>
<xml_diff>
--- a/templates/Plantilla de Pagos de Estudiantes - IUAF.xlsx
+++ b/templates/Plantilla de Pagos de Estudiantes - IUAF.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\1171566\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\1171566\Documents\vscode\iuaf-pro-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D998B60-AEC4-4CFB-B1FD-CA657E01F295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BEE8F2F-87CE-4717-9409-0D69B6FC6AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{627E0FEB-C1EB-4370-9A2E-554A4FD71355}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Concepto</t>
   </si>
@@ -57,16 +57,26 @@
   </si>
   <si>
     <t>ARIAS CASTILLO JUAN</t>
+  </si>
+  <si>
+    <t>No. de autorización</t>
+  </si>
+  <si>
+    <t>Sede</t>
+  </si>
+  <si>
+    <t>Cancún</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +86,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -100,16 +117,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -442,48 +462,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B1477E6-C797-4C68-B73A-3574C804A631}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="42.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45931</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4">
+        <v>999999</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>1</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>581</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>6</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>